<commit_message>
Adopt visually checked P8 warning layout and bind current Office evidence
</commit_message>
<xml_diff>
--- a/tools/candidates/remaining-batch-r3-20261018/checkpoint-working/P8/09-raschet-otrabotannoy-chasti-avansa.xlsx
+++ b/tools/candidates/remaining-batch-r3-20261018/checkpoint-working/P8/09-raschet-otrabotannoy-chasti-avansa.xlsx
@@ -1166,7 +1166,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="15">
         <f>IF(C6="","",ROW()-5)</f>
         <v/>
@@ -1188,7 +1188,7 @@
         <f>IF(E6="","",IF(F6="","не выбран статус",IF(I6+J6&gt;E6+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F6&lt;&gt;"подписан обеими сторонами",I6&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F6="подписан обеими сторонами",I6+J6=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F6&lt;&gt;"подписан обеими сторонами",G6=""),"Акт не подписан: укажите дату передачи.",IF(AND(F6&lt;&gt;"подписан обеими сторонами",H6=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="15">
         <f>IF(C7="","",ROW()-5)</f>
         <v/>
@@ -1210,7 +1210,7 @@
         <f>IF(E7="","",IF(F7="","не выбран статус",IF(I7+J7&gt;E7+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F7&lt;&gt;"подписан обеими сторонами",I7&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F7="подписан обеими сторонами",I7+J7=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F7&lt;&gt;"подписан обеими сторонами",G7=""),"Акт не подписан: укажите дату передачи.",IF(AND(F7&lt;&gt;"подписан обеими сторонами",H7=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="45" customHeight="1">
       <c r="A8" s="15">
         <f>IF(C8="","",ROW()-5)</f>
         <v/>
@@ -1232,7 +1232,7 @@
         <f>IF(E8="","",IF(F8="","не выбран статус",IF(I8+J8&gt;E8+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F8&lt;&gt;"подписан обеими сторонами",I8&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F8="подписан обеими сторонами",I8+J8=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F8&lt;&gt;"подписан обеими сторонами",G8=""),"Акт не подписан: укажите дату передачи.",IF(AND(F8&lt;&gt;"подписан обеими сторонами",H8=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="15">
         <f>IF(C9="","",ROW()-5)</f>
         <v/>
@@ -1254,7 +1254,7 @@
         <f>IF(E9="","",IF(F9="","не выбран статус",IF(I9+J9&gt;E9+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F9&lt;&gt;"подписан обеими сторонами",I9&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F9="подписан обеими сторонами",I9+J9=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F9&lt;&gt;"подписан обеими сторонами",G9=""),"Акт не подписан: укажите дату передачи.",IF(AND(F9&lt;&gt;"подписан обеими сторонами",H9=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="15">
         <f>IF(C10="","",ROW()-5)</f>
         <v/>
@@ -1276,7 +1276,7 @@
         <f>IF(E10="","",IF(F10="","не выбран статус",IF(I10+J10&gt;E10+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F10&lt;&gt;"подписан обеими сторонами",I10&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F10="подписан обеими сторонами",I10+J10=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F10&lt;&gt;"подписан обеими сторонами",G10=""),"Акт не подписан: укажите дату передачи.",IF(AND(F10&lt;&gt;"подписан обеими сторонами",H10=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="15">
         <f>IF(C11="","",ROW()-5)</f>
         <v/>
@@ -1298,7 +1298,7 @@
         <f>IF(E11="","",IF(F11="","не выбран статус",IF(I11+J11&gt;E11+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F11&lt;&gt;"подписан обеими сторонами",I11&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F11="подписан обеими сторонами",I11+J11=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F11&lt;&gt;"подписан обеими сторонами",G11=""),"Акт не подписан: укажите дату передачи.",IF(AND(F11&lt;&gt;"подписан обеими сторонами",H11=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="15">
         <f>IF(C12="","",ROW()-5)</f>
         <v/>
@@ -1320,7 +1320,7 @@
         <f>IF(E12="","",IF(F12="","не выбран статус",IF(I12+J12&gt;E12+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F12&lt;&gt;"подписан обеими сторонами",I12&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F12="подписан обеими сторонами",I12+J12=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F12&lt;&gt;"подписан обеими сторонами",G12=""),"Акт не подписан: укажите дату передачи.",IF(AND(F12&lt;&gt;"подписан обеими сторонами",H12=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="15">
         <f>IF(C13="","",ROW()-5)</f>
         <v/>
@@ -1342,7 +1342,7 @@
         <f>IF(E13="","",IF(F13="","не выбран статус",IF(I13+J13&gt;E13+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F13&lt;&gt;"подписан обеими сторонами",I13&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F13="подписан обеими сторонами",I13+J13=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F13&lt;&gt;"подписан обеими сторонами",G13=""),"Акт не подписан: укажите дату передачи.",IF(AND(F13&lt;&gt;"подписан обеими сторонами",H13=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="15">
         <f>IF(C14="","",ROW()-5)</f>
         <v/>
@@ -1364,7 +1364,7 @@
         <f>IF(E14="","",IF(F14="","не выбран статус",IF(I14+J14&gt;E14+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F14&lt;&gt;"подписан обеими сторонами",I14&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F14="подписан обеими сторонами",I14+J14=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F14&lt;&gt;"подписан обеими сторонами",G14=""),"Акт не подписан: укажите дату передачи.",IF(AND(F14&lt;&gt;"подписан обеими сторонами",H14=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="15">
         <f>IF(C15="","",ROW()-5)</f>
         <v/>
@@ -1386,7 +1386,7 @@
         <f>IF(E15="","",IF(F15="","не выбран статус",IF(I15+J15&gt;E15+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F15&lt;&gt;"подписан обеими сторонами",I15&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F15="подписан обеими сторонами",I15+J15=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F15&lt;&gt;"подписан обеими сторонами",G15=""),"Акт не подписан: укажите дату передачи.",IF(AND(F15&lt;&gt;"подписан обеими сторонами",H15=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="45" customHeight="1">
       <c r="A16" s="15">
         <f>IF(C16="","",ROW()-5)</f>
         <v/>
@@ -1408,7 +1408,7 @@
         <f>IF(E16="","",IF(F16="","не выбран статус",IF(I16+J16&gt;E16+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F16&lt;&gt;"подписан обеими сторонами",I16&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F16="подписан обеими сторонами",I16+J16=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F16&lt;&gt;"подписан обеими сторонами",G16=""),"Акт не подписан: укажите дату передачи.",IF(AND(F16&lt;&gt;"подписан обеими сторонами",H16=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="15">
         <f>IF(C17="","",ROW()-5)</f>
         <v/>
@@ -1430,7 +1430,7 @@
         <f>IF(E17="","",IF(F17="","не выбран статус",IF(I17+J17&gt;E17+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F17&lt;&gt;"подписан обеими сторонами",I17&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F17="подписан обеими сторонами",I17+J17=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F17&lt;&gt;"подписан обеими сторонами",G17=""),"Акт не подписан: укажите дату передачи.",IF(AND(F17&lt;&gt;"подписан обеими сторонами",H17=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="45" customHeight="1">
       <c r="A18" s="15">
         <f>IF(C18="","",ROW()-5)</f>
         <v/>
@@ -1452,7 +1452,7 @@
         <f>IF(E18="","",IF(F18="","не выбран статус",IF(I18+J18&gt;E18+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F18&lt;&gt;"подписан обеими сторонами",I18&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F18="подписан обеими сторонами",I18+J18=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F18&lt;&gt;"подписан обеими сторонами",G18=""),"Акт не подписан: укажите дату передачи.",IF(AND(F18&lt;&gt;"подписан обеими сторонами",H18=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="45" customHeight="1">
       <c r="A19" s="15">
         <f>IF(C19="","",ROW()-5)</f>
         <v/>
@@ -1474,7 +1474,7 @@
         <f>IF(E19="","",IF(F19="","не выбран статус",IF(I19+J19&gt;E19+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F19&lt;&gt;"подписан обеими сторонами",I19&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F19="подписан обеими сторонами",I19+J19=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F19&lt;&gt;"подписан обеими сторонами",G19=""),"Акт не подписан: укажите дату передачи.",IF(AND(F19&lt;&gt;"подписан обеими сторонами",H19=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="45" customHeight="1">
       <c r="A20" s="15">
         <f>IF(C20="","",ROW()-5)</f>
         <v/>
@@ -1496,7 +1496,7 @@
         <f>IF(E20="","",IF(F20="","не выбран статус",IF(I20+J20&gt;E20+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F20&lt;&gt;"подписан обеими сторонами",I20&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F20="подписан обеими сторонами",I20+J20=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F20&lt;&gt;"подписан обеими сторонами",G20=""),"Акт не подписан: укажите дату передачи.",IF(AND(F20&lt;&gt;"подписан обеими сторонами",H20=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="45" customHeight="1">
       <c r="A21" s="15">
         <f>IF(C21="","",ROW()-5)</f>
         <v/>
@@ -1518,7 +1518,7 @@
         <f>IF(E21="","",IF(F21="","не выбран статус",IF(I21+J21&gt;E21+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F21&lt;&gt;"подписан обеими сторонами",I21&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F21="подписан обеими сторонами",I21+J21=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F21&lt;&gt;"подписан обеими сторонами",G21=""),"Акт не подписан: укажите дату передачи.",IF(AND(F21&lt;&gt;"подписан обеими сторонами",H21=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="15">
         <f>IF(C22="","",ROW()-5)</f>
         <v/>
@@ -1540,7 +1540,7 @@
         <f>IF(E22="","",IF(F22="","не выбран статус",IF(I22+J22&gt;E22+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F22&lt;&gt;"подписан обеими сторонами",I22&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F22="подписан обеими сторонами",I22+J22=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F22&lt;&gt;"подписан обеими сторонами",G22=""),"Акт не подписан: укажите дату передачи.",IF(AND(F22&lt;&gt;"подписан обеими сторонами",H22=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="45" customHeight="1">
       <c r="A23" s="15">
         <f>IF(C23="","",ROW()-5)</f>
         <v/>
@@ -1562,7 +1562,7 @@
         <f>IF(E23="","",IF(F23="","не выбран статус",IF(I23+J23&gt;E23+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F23&lt;&gt;"подписан обеими сторонами",I23&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F23="подписан обеими сторонами",I23+J23=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F23&lt;&gt;"подписан обеими сторонами",G23=""),"Акт не подписан: укажите дату передачи.",IF(AND(F23&lt;&gt;"подписан обеими сторонами",H23=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="45" customHeight="1">
       <c r="A24" s="15">
         <f>IF(C24="","",ROW()-5)</f>
         <v/>
@@ -1584,7 +1584,7 @@
         <f>IF(E24="","",IF(F24="","не выбран статус",IF(I24+J24&gt;E24+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F24&lt;&gt;"подписан обеими сторонами",I24&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F24="подписан обеими сторонами",I24+J24=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F24&lt;&gt;"подписан обеими сторонами",G24=""),"Акт не подписан: укажите дату передачи.",IF(AND(F24&lt;&gt;"подписан обеими сторонами",H24=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="45" customHeight="1">
       <c r="A25" s="15">
         <f>IF(C25="","",ROW()-5)</f>
         <v/>
@@ -1606,7 +1606,7 @@
         <f>IF(E25="","",IF(F25="","не выбран статус",IF(I25+J25&gt;E25+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F25&lt;&gt;"подписан обеими сторонами",I25&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F25="подписан обеими сторонами",I25+J25=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F25&lt;&gt;"подписан обеими сторонами",G25=""),"Акт не подписан: укажите дату передачи.",IF(AND(F25&lt;&gt;"подписан обеими сторонами",H25=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="45" customHeight="1">
       <c r="A26" s="15">
         <f>IF(C26="","",ROW()-5)</f>
         <v/>
@@ -1628,7 +1628,7 @@
         <f>IF(E26="","",IF(F26="","не выбран статус",IF(I26+J26&gt;E26+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F26&lt;&gt;"подписан обеими сторонами",I26&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F26="подписан обеими сторонами",I26+J26=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F26&lt;&gt;"подписан обеими сторонами",G26=""),"Акт не подписан: укажите дату передачи.",IF(AND(F26&lt;&gt;"подписан обеими сторонами",H26=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="45" customHeight="1">
       <c r="A27" s="15">
         <f>IF(C27="","",ROW()-5)</f>
         <v/>
@@ -1650,7 +1650,7 @@
         <f>IF(E27="","",IF(F27="","не выбран статус",IF(I27+J27&gt;E27+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F27&lt;&gt;"подписан обеими сторонами",I27&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F27="подписан обеими сторонами",I27+J27=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F27&lt;&gt;"подписан обеими сторонами",G27=""),"Акт не подписан: укажите дату передачи.",IF(AND(F27&lt;&gt;"подписан обеими сторонами",H27=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="45" customHeight="1">
       <c r="A28" s="15">
         <f>IF(C28="","",ROW()-5)</f>
         <v/>
@@ -1672,7 +1672,7 @@
         <f>IF(E28="","",IF(F28="","не выбран статус",IF(I28+J28&gt;E28+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F28&lt;&gt;"подписан обеими сторонами",I28&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F28="подписан обеими сторонами",I28+J28=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F28&lt;&gt;"подписан обеими сторонами",G28=""),"Акт не подписан: укажите дату передачи.",IF(AND(F28&lt;&gt;"подписан обеими сторонами",H28=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="45" customHeight="1">
       <c r="A29" s="15">
         <f>IF(C29="","",ROW()-5)</f>
         <v/>
@@ -1694,7 +1694,7 @@
         <f>IF(E29="","",IF(F29="","не выбран статус",IF(I29+J29&gt;E29+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F29&lt;&gt;"подписан обеими сторонами",I29&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F29="подписан обеими сторонами",I29+J29=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F29&lt;&gt;"подписан обеими сторонами",G29=""),"Акт не подписан: укажите дату передачи.",IF(AND(F29&lt;&gt;"подписан обеими сторонами",H29=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="45" customHeight="1">
       <c r="A30" s="15">
         <f>IF(C30="","",ROW()-5)</f>
         <v/>
@@ -1716,7 +1716,7 @@
         <f>IF(E30="","",IF(F30="","не выбран статус",IF(I30+J30&gt;E30+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F30&lt;&gt;"подписан обеими сторонами",I30&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F30="подписан обеими сторонами",I30+J30=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F30&lt;&gt;"подписан обеими сторонами",G30=""),"Акт не подписан: укажите дату передачи.",IF(AND(F30&lt;&gt;"подписан обеими сторонами",H30=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="45" customHeight="1">
       <c r="A31" s="15">
         <f>IF(C31="","",ROW()-5)</f>
         <v/>
@@ -1738,7 +1738,7 @@
         <f>IF(E31="","",IF(F31="","не выбран статус",IF(I31+J31&gt;E31+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F31&lt;&gt;"подписан обеими сторонами",I31&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F31="подписан обеими сторонами",I31+J31=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F31&lt;&gt;"подписан обеими сторонами",G31=""),"Акт не подписан: укажите дату передачи.",IF(AND(F31&lt;&gt;"подписан обеими сторонами",H31=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="45" customHeight="1">
       <c r="A32" s="15">
         <f>IF(C32="","",ROW()-5)</f>
         <v/>
@@ -1760,7 +1760,7 @@
         <f>IF(E32="","",IF(F32="","не выбран статус",IF(I32+J32&gt;E32+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F32&lt;&gt;"подписан обеими сторонами",I32&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F32="подписан обеими сторонами",I32+J32=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F32&lt;&gt;"подписан обеими сторонами",G32=""),"Акт не подписан: укажите дату передачи.",IF(AND(F32&lt;&gt;"подписан обеими сторонами",H32=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="45" customHeight="1">
       <c r="A33" s="15">
         <f>IF(C33="","",ROW()-5)</f>
         <v/>
@@ -1782,7 +1782,7 @@
         <f>IF(E33="","",IF(F33="","не выбран статус",IF(I33+J33&gt;E33+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F33&lt;&gt;"подписан обеими сторонами",I33&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F33="подписан обеими сторонами",I33+J33=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F33&lt;&gt;"подписан обеими сторонами",G33=""),"Акт не подписан: укажите дату передачи.",IF(AND(F33&lt;&gt;"подписан обеими сторонами",H33=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="45" customHeight="1">
       <c r="A34" s="15">
         <f>IF(C34="","",ROW()-5)</f>
         <v/>
@@ -1804,7 +1804,7 @@
         <f>IF(E34="","",IF(F34="","не выбран статус",IF(I34+J34&gt;E34+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F34&lt;&gt;"подписан обеими сторонами",I34&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F34="подписан обеими сторонами",I34+J34=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F34&lt;&gt;"подписан обеими сторонами",G34=""),"Акт не подписан: укажите дату передачи.",IF(AND(F34&lt;&gt;"подписан обеими сторонами",H34=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="45" customHeight="1">
       <c r="A35" s="15">
         <f>IF(C35="","",ROW()-5)</f>
         <v/>
@@ -1826,7 +1826,7 @@
         <f>IF(E35="","",IF(F35="","не выбран статус",IF(I35+J35&gt;E35+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F35&lt;&gt;"подписан обеими сторонами",I35&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F35="подписан обеими сторонами",I35+J35=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F35&lt;&gt;"подписан обеими сторонами",G35=""),"Акт не подписан: укажите дату передачи.",IF(AND(F35&lt;&gt;"подписан обеими сторонами",H35=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="45" customHeight="1">
       <c r="A36" s="15">
         <f>IF(C36="","",ROW()-5)</f>
         <v/>
@@ -1848,7 +1848,7 @@
         <f>IF(E36="","",IF(F36="","не выбран статус",IF(I36+J36&gt;E36+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F36&lt;&gt;"подписан обеими сторонами",I36&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F36="подписан обеими сторонами",I36+J36=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F36&lt;&gt;"подписан обеими сторонами",G36=""),"Акт не подписан: укажите дату передачи.",IF(AND(F36&lt;&gt;"подписан обеими сторонами",H36=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="45" customHeight="1">
       <c r="A37" s="15">
         <f>IF(C37="","",ROW()-5)</f>
         <v/>
@@ -1870,7 +1870,7 @@
         <f>IF(E37="","",IF(F37="","не выбран статус",IF(I37+J37&gt;E37+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F37&lt;&gt;"подписан обеими сторонами",I37&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F37="подписан обеими сторонами",I37+J37=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F37&lt;&gt;"подписан обеими сторонами",G37=""),"Акт не подписан: укажите дату передачи.",IF(AND(F37&lt;&gt;"подписан обеими сторонами",H37=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="45" customHeight="1">
       <c r="A38" s="15">
         <f>IF(C38="","",ROW()-5)</f>
         <v/>
@@ -1892,7 +1892,7 @@
         <f>IF(E38="","",IF(F38="","не выбран статус",IF(I38+J38&gt;E38+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F38&lt;&gt;"подписан обеими сторонами",I38&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F38="подписан обеими сторонами",I38+J38=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F38&lt;&gt;"подписан обеими сторонами",G38=""),"Акт не подписан: укажите дату передачи.",IF(AND(F38&lt;&gt;"подписан обеими сторонами",H38=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="45" customHeight="1">
       <c r="A39" s="15">
         <f>IF(C39="","",ROW()-5)</f>
         <v/>
@@ -1914,7 +1914,7 @@
         <f>IF(E39="","",IF(F39="","не выбран статус",IF(I39+J39&gt;E39+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F39&lt;&gt;"подписан обеими сторонами",I39&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F39="подписан обеими сторонами",I39+J39=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F39&lt;&gt;"подписан обеими сторонами",G39=""),"Акт не подписан: укажите дату передачи.",IF(AND(F39&lt;&gt;"подписан обеими сторонами",H39=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="45" customHeight="1">
       <c r="A40" s="15">
         <f>IF(C40="","",ROW()-5)</f>
         <v/>
@@ -1936,7 +1936,7 @@
         <f>IF(E40="","",IF(F40="","не выбран статус",IF(I40+J40&gt;E40+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F40&lt;&gt;"подписан обеими сторонами",I40&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F40="подписан обеими сторонами",I40+J40=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F40&lt;&gt;"подписан обеими сторонами",G40=""),"Акт не подписан: укажите дату передачи.",IF(AND(F40&lt;&gt;"подписан обеими сторонами",H40=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="45" customHeight="1">
       <c r="A41" s="15">
         <f>IF(C41="","",ROW()-5)</f>
         <v/>
@@ -1958,7 +1958,7 @@
         <f>IF(E41="","",IF(F41="","не выбран статус",IF(I41+J41&gt;E41+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F41&lt;&gt;"подписан обеими сторонами",I41&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F41="подписан обеими сторонами",I41+J41=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F41&lt;&gt;"подписан обеими сторонами",G41=""),"Акт не подписан: укажите дату передачи.",IF(AND(F41&lt;&gt;"подписан обеими сторонами",H41=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="45" customHeight="1">
       <c r="A42" s="15">
         <f>IF(C42="","",ROW()-5)</f>
         <v/>
@@ -1980,7 +1980,7 @@
         <f>IF(E42="","",IF(F42="","не выбран статус",IF(I42+J42&gt;E42+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F42&lt;&gt;"подписан обеими сторонами",I42&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F42="подписан обеими сторонами",I42+J42=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F42&lt;&gt;"подписан обеими сторонами",G42=""),"Акт не подписан: укажите дату передачи.",IF(AND(F42&lt;&gt;"подписан обеими сторонами",H42=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="45" customHeight="1">
       <c r="A43" s="15">
         <f>IF(C43="","",ROW()-5)</f>
         <v/>
@@ -2002,7 +2002,7 @@
         <f>IF(E43="","",IF(F43="","не выбран статус",IF(I43+J43&gt;E43+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F43&lt;&gt;"подписан обеими сторонами",I43&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F43="подписан обеими сторонами",I43+J43=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F43&lt;&gt;"подписан обеими сторонами",G43=""),"Акт не подписан: укажите дату передачи.",IF(AND(F43&lt;&gt;"подписан обеими сторонами",H43=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="45" customHeight="1">
       <c r="A44" s="15">
         <f>IF(C44="","",ROW()-5)</f>
         <v/>
@@ -2024,7 +2024,7 @@
         <f>IF(E44="","",IF(F44="","не выбран статус",IF(I44+J44&gt;E44+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F44&lt;&gt;"подписан обеими сторонами",I44&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F44="подписан обеими сторонами",I44+J44=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F44&lt;&gt;"подписан обеими сторонами",G44=""),"Акт не подписан: укажите дату передачи.",IF(AND(F44&lt;&gt;"подписан обеими сторонами",H44=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="45" customHeight="1">
       <c r="A45" s="15">
         <f>IF(C45="","",ROW()-5)</f>
         <v/>
@@ -2182,9 +2182,7 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="25" min="0" max="16383" man="1"/>
-  </rowBreaks>
+  <rowBreaks count="0" manualBreakCount="0"/>
 </worksheet>
 </file>
 
@@ -2257,7 +2255,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="15">
         <f>IF(C6="","",ROW()-5)</f>
         <v/>
@@ -2271,7 +2269,7 @@
         <f>IF(D6="","",IF(B6="","не выбрано основание",IF(E6="","ОШИБКА: сумма без подтверждающего документа",IF(F6="","не указано, подписан ли документ второй стороной",IF(F6="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="15">
         <f>IF(C7="","",ROW()-5)</f>
         <v/>
@@ -2285,7 +2283,7 @@
         <f>IF(D7="","",IF(B7="","не выбрано основание",IF(E7="","ОШИБКА: сумма без подтверждающего документа",IF(F7="","не указано, подписан ли документ второй стороной",IF(F7="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="45" customHeight="1">
       <c r="A8" s="15">
         <f>IF(C8="","",ROW()-5)</f>
         <v/>
@@ -2299,7 +2297,7 @@
         <f>IF(D8="","",IF(B8="","не выбрано основание",IF(E8="","ОШИБКА: сумма без подтверждающего документа",IF(F8="","не указано, подписан ли документ второй стороной",IF(F8="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="15">
         <f>IF(C9="","",ROW()-5)</f>
         <v/>
@@ -2313,7 +2311,7 @@
         <f>IF(D9="","",IF(B9="","не выбрано основание",IF(E9="","ОШИБКА: сумма без подтверждающего документа",IF(F9="","не указано, подписан ли документ второй стороной",IF(F9="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="15">
         <f>IF(C10="","",ROW()-5)</f>
         <v/>
@@ -2327,7 +2325,7 @@
         <f>IF(D10="","",IF(B10="","не выбрано основание",IF(E10="","ОШИБКА: сумма без подтверждающего документа",IF(F10="","не указано, подписан ли документ второй стороной",IF(F10="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="15">
         <f>IF(C11="","",ROW()-5)</f>
         <v/>
@@ -2341,7 +2339,7 @@
         <f>IF(D11="","",IF(B11="","не выбрано основание",IF(E11="","ОШИБКА: сумма без подтверждающего документа",IF(F11="","не указано, подписан ли документ второй стороной",IF(F11="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="15">
         <f>IF(C12="","",ROW()-5)</f>
         <v/>
@@ -2355,7 +2353,7 @@
         <f>IF(D12="","",IF(B12="","не выбрано основание",IF(E12="","ОШИБКА: сумма без подтверждающего документа",IF(F12="","не указано, подписан ли документ второй стороной",IF(F12="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="15">
         <f>IF(C13="","",ROW()-5)</f>
         <v/>
@@ -2369,7 +2367,7 @@
         <f>IF(D13="","",IF(B13="","не выбрано основание",IF(E13="","ОШИБКА: сумма без подтверждающего документа",IF(F13="","не указано, подписан ли документ второй стороной",IF(F13="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="15">
         <f>IF(C14="","",ROW()-5)</f>
         <v/>
@@ -2383,7 +2381,7 @@
         <f>IF(D14="","",IF(B14="","не выбрано основание",IF(E14="","ОШИБКА: сумма без подтверждающего документа",IF(F14="","не указано, подписан ли документ второй стороной",IF(F14="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="15">
         <f>IF(C15="","",ROW()-5)</f>
         <v/>
@@ -2397,7 +2395,7 @@
         <f>IF(D15="","",IF(B15="","не выбрано основание",IF(E15="","ОШИБКА: сумма без подтверждающего документа",IF(F15="","не указано, подписан ли документ второй стороной",IF(F15="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="45" customHeight="1">
       <c r="A16" s="15">
         <f>IF(C16="","",ROW()-5)</f>
         <v/>
@@ -2411,7 +2409,7 @@
         <f>IF(D16="","",IF(B16="","не выбрано основание",IF(E16="","ОШИБКА: сумма без подтверждающего документа",IF(F16="","не указано, подписан ли документ второй стороной",IF(F16="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="15">
         <f>IF(C17="","",ROW()-5)</f>
         <v/>
@@ -2425,7 +2423,7 @@
         <f>IF(D17="","",IF(B17="","не выбрано основание",IF(E17="","ОШИБКА: сумма без подтверждающего документа",IF(F17="","не указано, подписан ли документ второй стороной",IF(F17="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="45" customHeight="1">
       <c r="A18" s="15">
         <f>IF(C18="","",ROW()-5)</f>
         <v/>
@@ -2439,7 +2437,7 @@
         <f>IF(D18="","",IF(B18="","не выбрано основание",IF(E18="","ОШИБКА: сумма без подтверждающего документа",IF(F18="","не указано, подписан ли документ второй стороной",IF(F18="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="45" customHeight="1">
       <c r="A19" s="15">
         <f>IF(C19="","",ROW()-5)</f>
         <v/>
@@ -2453,7 +2451,7 @@
         <f>IF(D19="","",IF(B19="","не выбрано основание",IF(E19="","ОШИБКА: сумма без подтверждающего документа",IF(F19="","не указано, подписан ли документ второй стороной",IF(F19="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="45" customHeight="1">
       <c r="A20" s="15">
         <f>IF(C20="","",ROW()-5)</f>
         <v/>
@@ -2467,7 +2465,7 @@
         <f>IF(D20="","",IF(B20="","не выбрано основание",IF(E20="","ОШИБКА: сумма без подтверждающего документа",IF(F20="","не указано, подписан ли документ второй стороной",IF(F20="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="45" customHeight="1">
       <c r="A21" s="15">
         <f>IF(C21="","",ROW()-5)</f>
         <v/>
@@ -2481,7 +2479,7 @@
         <f>IF(D21="","",IF(B21="","не выбрано основание",IF(E21="","ОШИБКА: сумма без подтверждающего документа",IF(F21="","не указано, подписан ли документ второй стороной",IF(F21="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="15">
         <f>IF(C22="","",ROW()-5)</f>
         <v/>
@@ -2495,7 +2493,7 @@
         <f>IF(D22="","",IF(B22="","не выбрано основание",IF(E22="","ОШИБКА: сумма без подтверждающего документа",IF(F22="","не указано, подписан ли документ второй стороной",IF(F22="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="45" customHeight="1">
       <c r="A23" s="15">
         <f>IF(C23="","",ROW()-5)</f>
         <v/>
@@ -2509,7 +2507,7 @@
         <f>IF(D23="","",IF(B23="","не выбрано основание",IF(E23="","ОШИБКА: сумма без подтверждающего документа",IF(F23="","не указано, подписан ли документ второй стороной",IF(F23="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="45" customHeight="1">
       <c r="A24" s="15">
         <f>IF(C24="","",ROW()-5)</f>
         <v/>
@@ -2523,7 +2521,7 @@
         <f>IF(D24="","",IF(B24="","не выбрано основание",IF(E24="","ОШИБКА: сумма без подтверждающего документа",IF(F24="","не указано, подписан ли документ второй стороной",IF(F24="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="45" customHeight="1">
       <c r="A25" s="15">
         <f>IF(C25="","",ROW()-5)</f>
         <v/>
@@ -2537,7 +2535,7 @@
         <f>IF(D25="","",IF(B25="","не выбрано основание",IF(E25="","ОШИБКА: сумма без подтверждающего документа",IF(F25="","не указано, подписан ли документ второй стороной",IF(F25="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="45" customHeight="1">
       <c r="A26" s="15">
         <f>IF(C26="","",ROW()-5)</f>
         <v/>
@@ -2551,7 +2549,7 @@
         <f>IF(D26="","",IF(B26="","не выбрано основание",IF(E26="","ОШИБКА: сумма без подтверждающего документа",IF(F26="","не указано, подписан ли документ второй стороной",IF(F26="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="45" customHeight="1">
       <c r="A27" s="15">
         <f>IF(C27="","",ROW()-5)</f>
         <v/>
@@ -2565,7 +2563,7 @@
         <f>IF(D27="","",IF(B27="","не выбрано основание",IF(E27="","ОШИБКА: сумма без подтверждающего документа",IF(F27="","не указано, подписан ли документ второй стороной",IF(F27="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="45" customHeight="1">
       <c r="A28" s="15">
         <f>IF(C28="","",ROW()-5)</f>
         <v/>
@@ -2579,7 +2577,7 @@
         <f>IF(D28="","",IF(B28="","не выбрано основание",IF(E28="","ОШИБКА: сумма без подтверждающего документа",IF(F28="","не указано, подписан ли документ второй стороной",IF(F28="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="45" customHeight="1">
       <c r="A29" s="15">
         <f>IF(C29="","",ROW()-5)</f>
         <v/>
@@ -2593,7 +2591,7 @@
         <f>IF(D29="","",IF(B29="","не выбрано основание",IF(E29="","ОШИБКА: сумма без подтверждающего документа",IF(F29="","не указано, подписан ли документ второй стороной",IF(F29="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="45" customHeight="1">
       <c r="A30" s="15">
         <f>IF(C30="","",ROW()-5)</f>
         <v/>
@@ -2730,8 +2728,9 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="21" min="0" max="16383" man="1"/>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="15" min="0" max="16383" man="1"/>
+    <brk id="25" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>

</xml_diff>